<commit_message>
docs(pruebas): ejecutar los casos funcionales contra la aplicacion desplegada
Los pasos apuntaban a http://localhost:4200, que solo existe en la maquina de
quien desarrolla. Ahora el paso 1 de cada caso entra a
https://gen-ova-frontend.vercel.app, que es la aplicacion que el lector puede
abrir para reproducir la prueba.

El caso 2.3 se reescribio ademas de fondo: comprobaba la validacion de fase y
tipo de recurso desde /docs (Swagger) del backend local, pero la documentacion
interactiva esta deshabilitada en produccion (ENV=production apaga docs_url).
Ahora la comprobacion se hace desde la consola del navegador con la sesion ya
iniciada, contra la API desplegada, y el motivo queda escrito en el comentario
del caso.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pruebas/Casos de prueba - Pruebas Funcionales.xlsx
+++ b/docs/pruebas/Casos de prueba - Pruebas Funcionales.xlsx
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Método: tabla de decisiones fase × tipo de recurso contra el catálogo RECURSOS_META.</t>
+          <t>Método: tabla de decisiones fase × tipo de recurso contra el catálogo RECURSOS_META. La documentación interactiva (/docs) está deshabilitada en producción, así que la comprobación se hace desde la consola del navegador con la sesión activa.</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a la aplicación en http://localhost:4200. La aplicación redirige a la pantalla de inicio de sesión (/login) por no haber sesión activa.</t>
+          <t>Abrir el navegador e ingresar a la aplicación desplegada en https://gen-ova-frontend.vercel.app. La aplicación redirige a la pantalla de inicio de sesión (https://gen-ova-frontend.vercel.app/login) por no haber sesión activa.</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a http://localhost:4200/login.</t>
+          <t>Abrir el navegador e ingresar a https://gen-ova-frontend.vercel.app/login.</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a http://localhost:4200/login.</t>
+          <t>Abrir el navegador e ingresar a https://gen-ova-frontend.vercel.app/login.</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="B58" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a http://localhost:4200/login.</t>
+          <t>Abrir el navegador e ingresar a https://gen-ova-frontend.vercel.app/login.</t>
         </is>
       </c>
       <c r="C58" s="18" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="B73" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con «user@genova.ai» / «user1234password».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con «user@genova.ai» / «user1234password».</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B87" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con una cuenta de prueba creada para este caso.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con una cuenta de prueba creada para este caso.</t>
         </is>
       </c>
       <c r="C87" s="18" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B103" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a http://localhost:4200/reset-password SIN el parámetro token en la URL.</t>
+          <t>Abrir el navegador e ingresar a https://gen-ova-frontend.vercel.app/reset-password SIN el parámetro token en la URL.</t>
         </is>
       </c>
       <c r="C103" s="18" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="B104" s="18" t="inlineStr">
         <is>
-          <t>Ingresar ahora a http://localhost:4200/reset-password?token=token-de-prueba-invalido.</t>
+          <t>Ingresar ahora a https://gen-ova-frontend.vercel.app/reset-password?token=token-de-prueba-invalido.</t>
         </is>
       </c>
       <c r="C104" s="18" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B118" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador e ingresar a http://localhost:4200/verify-email SIN el parámetro token en la URL.</t>
+          <t>Abrir el navegador e ingresar a https://gen-ova-frontend.vercel.app/verify-email SIN el parámetro token en la URL.</t>
         </is>
       </c>
       <c r="C118" s="18" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="B119" s="18" t="inlineStr">
         <is>
-          <t>Ingresar a http://localhost:4200/verify-email?token=token-de-prueba-invalido.</t>
+          <t>Ingresar a https://gen-ova-frontend.vercel.app/verify-email?token=token-de-prueba-invalido.</t>
         </is>
       </c>
       <c r="C119" s="18" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con «user@genova.ai» / «user1234password».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con «user@genova.ai» / «user1234password».</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a /crear.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a /crear.</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a /crear.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a /crear.</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -5055,12 +5055,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse para obtener la cookie de sesión.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con «user@genova.ai» / «user1234password».</t>
         </is>
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>Autentica y emite la cookie httpOnly genova_token.</t>
+          <t>Autentica y el backend emite la cookie httpOnly genova_token para el dominio de la API.</t>
         </is>
       </c>
       <c r="D57" s="32" t="inlineStr">
@@ -5077,12 +5077,12 @@
       </c>
       <c r="B58" s="18" t="inlineStr">
         <is>
-          <t>Abrir la documentación interactiva del backend en http://localhost:8000/docs y desplegar «Generación → POST /api/jobs».</t>
+          <t>Abrir las herramientas de desarrollo del navegador (F12) y situarse en la pestaña Consola, sin salir del dominio de la aplicación.</t>
         </is>
       </c>
       <c r="C58" s="18" t="inlineStr">
         <is>
-          <t>Muestra la ficha del endpoint con su esquema de petición.</t>
+          <t>La consola queda lista para lanzar peticiones con la sesión ya iniciada.</t>
         </is>
       </c>
       <c r="D58" s="32" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>Pulsar «Try it out» y enviar un cuerpo con una combinación inválida: recurso «Lectura Interactiva» dentro de la fase «engage».</t>
+          <t>Enviar una petición a POST /api/jobs de la API desplegada con una combinación inválida: el recurso «Lectura Interactiva» dentro de la fase «engage».</t>
         </is>
       </c>
       <c r="C59" s="18" t="inlineStr">
@@ -5121,12 +5121,12 @@
       </c>
       <c r="B60" s="18" t="inlineStr">
         <is>
-          <t>Repetir el envío con la combinación válida: «Lectura Interactiva» en la fase «explore».</t>
+          <t>Repetir la petición con la combinación válida: «Lectura Interactiva» en la fase «explore».</t>
         </is>
       </c>
       <c r="C60" s="18" t="inlineStr">
         <is>
-          <t>El backend responde HTTP 202 y encola el trabajo con normalidad.</t>
+          <t>El backend responde HTTP 202 y encola el trabajo con normalidad, devolviendo su identificador.</t>
         </is>
       </c>
       <c r="D60" s="32" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>Consultar el estado del trabajo encolado en GET /api/jobs/{job_id}.</t>
+          <t>Consultar el estado de ese trabajo en GET /api/jobs/{job_id} con el identificador devuelto.</t>
         </is>
       </c>
       <c r="C61" s="18" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="B63" s="37" t="inlineStr">
         <is>
-          <t>Método: tabla de decisiones fase × tipo de recurso contra el catálogo RECURSOS_META.</t>
+          <t>Método: tabla de decisiones fase × tipo de recurso contra el catálogo RECURSOS_META. La documentación interactiva (/docs) está deshabilitada en producción, así que la comprobación se hace desde la consola del navegador con la sesión activa.</t>
         </is>
       </c>
       <c r="C63" s="41" t="n"/>
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B72" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a /crear.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a /crear.</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="B87" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse.</t>
         </is>
       </c>
       <c r="C87" s="18" t="inlineStr">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y abrir un OVA «Listo» desde «Mis OVAs».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y abrir un OVA «Listo» desde «Mis OVAs».</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse.</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="B52" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a «Mis OVAs».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a «Mis OVAs».</t>
         </is>
       </c>
       <c r="C52" s="18" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="B66" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a «Mis OVAs».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a «Mis OVAs».</t>
         </is>
       </c>
       <c r="C66" s="18" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B80" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y navegar a «Papelera».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y navegar a «Papelera».</t>
         </is>
       </c>
       <c r="C80" s="18" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con «admin@genova.ai» / «admin1234password».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con «admin@genova.ai» / «admin1234password».</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse como administrador.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse como administrador.</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse como administrador y navegar a /admin/roles.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse como administrador y navegar a /admin/roles.</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="B54" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con la cuenta SIN rol administrador «user@genova.ai».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con la cuenta SIN rol administrador «user@genova.ai».</t>
         </is>
       </c>
       <c r="C54" s="18" t="inlineStr">
@@ -8221,7 +8221,7 @@
       </c>
       <c r="B68" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse como administrador.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse como administrador.</t>
         </is>
       </c>
       <c r="C68" s="18" t="inlineStr">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="B82" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse como administrador y navegar a /models.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse como administrador y navegar a /models.</t>
         </is>
       </c>
       <c r="C82" s="18" t="inlineStr">
@@ -8688,7 +8688,7 @@
       </c>
       <c r="B97" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse como administrador.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse como administrador.</t>
         </is>
       </c>
       <c r="C97" s="18" t="inlineStr">
@@ -8932,7 +8932,7 @@
       </c>
       <c r="B112" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con una cuenta con permiso de analítica (administrador).</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con una cuenta con permiso de analítica (administrador).</t>
         </is>
       </c>
       <c r="C112" s="18" t="inlineStr">
@@ -9271,7 +9271,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y abrir las herramientas de desarrollo en la pestaña de red.</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y abrir las herramientas de desarrollo en la pestaña de red.</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login, autenticarse y descargar el paquete de un OVA «Listo» desde «Mis OVAs».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login, autenticarse y descargar el paquete de un OVA «Listo» desde «Mis OVAs».</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Abrir el navegador, ingresar a http://localhost:4200/login y autenticarse con «user@genova.ai» / «user1234password».</t>
+          <t>Abrir el navegador, ingresar a https://gen-ova-frontend.vercel.app/login y autenticarse con «user@genova.ai» / «user1234password».</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">

</xml_diff>